<commit_message>
added persistence of session_key when server shuts down
</commit_message>
<xml_diff>
--- a/src/serveur/1 - CONSERVER/Tests MCTS.xlsx
+++ b/src/serveur/1 - CONSERVER/Tests MCTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\src\serveur\1 - CONSERVER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4DE645-4CF3-4662-BDE1-A0BBEAD381F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84196853-F1AF-4F3C-9497-F6B9419EBA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{62420DB8-13EB-4D50-AF22-AC8AB6867586}"/>
   </bookViews>
@@ -339,9 +339,6 @@
     <t>(5,6) → (5,5)</t>
   </si>
   <si>
-    <t xml:space="preserve">Informations parfaites (tout le plateau de jeu est connu de l'IA) </t>
-  </si>
-  <si>
     <t>Informations imparfaites (les pièces de l'opposant ne sont pas connues de l'IA)</t>
   </si>
   <si>
@@ -358,6 +355,9 @@
   </si>
   <si>
     <t>Présence des meilleurs coups selon les itérations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informations parfaites (les pièces de l'opposant sont connues de l'IA) </t>
   </si>
 </sst>
 </file>
@@ -1250,8 +1250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB83B5AC-29A4-4763-B7BA-92B1F1A3FC5C}" name="Tableau1" displayName="Tableau1" ref="B6:H9" totalsRowShown="0" headerRowDxfId="29" dataDxfId="42">
-  <autoFilter ref="B6:H9" xr:uid="{BB83B5AC-29A4-4763-B7BA-92B1F1A3FC5C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BB83B5AC-29A4-4763-B7BA-92B1F1A3FC5C}" name="Tableau1" displayName="Tableau1" ref="B5:H8" totalsRowShown="0" headerRowDxfId="29" dataDxfId="42">
+  <autoFilter ref="B5:H8" xr:uid="{BB83B5AC-29A4-4763-B7BA-92B1F1A3FC5C}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{9C3463D2-929F-4FFD-B3E2-9BC649245AD8}" name="Budget" dataDxfId="45"/>
     <tableColumn id="2" xr3:uid="{EFE78F93-3878-4D8B-9551-71DA6E396EB5}" name="Exécutions" dataDxfId="44"/>
@@ -1266,8 +1266,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06E6C9D5-7376-492B-8904-3AB4EB51828F}" name="Tableau2" displayName="Tableau2" ref="B13:E17" totalsRowShown="0" headerRowDxfId="41" dataDxfId="36">
-  <autoFilter ref="B13:E17" xr:uid="{06E6C9D5-7376-492B-8904-3AB4EB51828F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06E6C9D5-7376-492B-8904-3AB4EB51828F}" name="Tableau2" displayName="Tableau2" ref="B12:E16" totalsRowShown="0" headerRowDxfId="41" dataDxfId="36">
+  <autoFilter ref="B12:E16" xr:uid="{06E6C9D5-7376-492B-8904-3AB4EB51828F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0FC10192-0187-47FA-9E60-FD0A6944FA13}" name="Indicateur" dataDxfId="40"/>
     <tableColumn id="2" xr3:uid="{E1A035C2-4A8C-480F-B7BE-7D5B8FF3385E}" name="500 → 2000" dataDxfId="39"/>
@@ -1279,8 +1279,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D2AEE367-4DA7-4035-B4FE-FF08D787A772}" name="Tableau3" displayName="Tableau3" ref="B21:D28" totalsRowShown="0" headerRowDxfId="35" dataDxfId="31">
-  <autoFilter ref="B21:D28" xr:uid="{D2AEE367-4DA7-4035-B4FE-FF08D787A772}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D2AEE367-4DA7-4035-B4FE-FF08D787A772}" name="Tableau3" displayName="Tableau3" ref="B20:D27" totalsRowShown="0" headerRowDxfId="35" dataDxfId="31">
+  <autoFilter ref="B20:D27" xr:uid="{D2AEE367-4DA7-4035-B4FE-FF08D787A772}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{43C10F74-441D-45BD-95BD-EAA6621EE7C4}" name="Budget" dataDxfId="34"/>
     <tableColumn id="2" xr3:uid="{BBFC201C-DD0E-4132-A1EC-D214CBCDB7E4}" name="Coup" dataDxfId="33"/>
@@ -1291,8 +1291,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{92F4D6DC-E8AD-42A4-A84A-8AA399205719}" name="Tableau5" displayName="Tableau5" ref="B35:I38" totalsRowShown="0" headerRowDxfId="30" dataDxfId="20">
-  <autoFilter ref="B35:I38" xr:uid="{92F4D6DC-E8AD-42A4-A84A-8AA399205719}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{92F4D6DC-E8AD-42A4-A84A-8AA399205719}" name="Tableau5" displayName="Tableau5" ref="B33:I36" totalsRowShown="0" headerRowDxfId="30" dataDxfId="20">
+  <autoFilter ref="B33:I36" xr:uid="{92F4D6DC-E8AD-42A4-A84A-8AA399205719}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{2D4FD578-FA2D-4384-9263-69A6F90BE3A1}" name="Budget" dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{A7D22749-5557-4516-AA5B-DAA2AD7A3818}" name="Exécutions" dataDxfId="27"/>
@@ -1308,8 +1308,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AF9F18BF-7207-4B21-987D-78E9EB107C14}" name="Tableau7" displayName="Tableau7" ref="B42:E46" totalsRowShown="0" headerRowDxfId="15" dataDxfId="10">
-  <autoFilter ref="B42:E46" xr:uid="{AF9F18BF-7207-4B21-987D-78E9EB107C14}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AF9F18BF-7207-4B21-987D-78E9EB107C14}" name="Tableau7" displayName="Tableau7" ref="B40:E44" totalsRowShown="0" headerRowDxfId="15" dataDxfId="10">
+  <autoFilter ref="B40:E44" xr:uid="{AF9F18BF-7207-4B21-987D-78E9EB107C14}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9EF471DF-8318-48B2-8FA8-9CA0250CBD6A}" name="Indicateur" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{AC7D058A-B01F-4CB9-94F4-8F489C7AEA48}" name="500 → 2000" dataDxfId="13"/>
@@ -1321,8 +1321,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{198CF64D-7923-49E2-AE1D-DAA85340DE69}" name="Tableau8" displayName="Tableau8" ref="B50:D59" totalsRowShown="0" headerRowDxfId="9" dataDxfId="5">
-  <autoFilter ref="B50:D59" xr:uid="{198CF64D-7923-49E2-AE1D-DAA85340DE69}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{198CF64D-7923-49E2-AE1D-DAA85340DE69}" name="Tableau8" displayName="Tableau8" ref="B48:D57" totalsRowShown="0" headerRowDxfId="9" dataDxfId="5">
+  <autoFilter ref="B48:D57" xr:uid="{198CF64D-7923-49E2-AE1D-DAA85340DE69}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{2C5C1F62-D80C-4C6C-9414-733C53707DC5}" name="Budget" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{E6C2E2D9-D347-4F47-9738-FEB5576497D6}" name="Coup" dataDxfId="7"/>
@@ -1333,8 +1333,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{18208E07-AE00-42BB-B6B8-7046468EAA03}" name="Tableau610" displayName="Tableau610" ref="G21:I26" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="G21:I26" xr:uid="{18208E07-AE00-42BB-B6B8-7046468EAA03}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{18208E07-AE00-42BB-B6B8-7046468EAA03}" name="Tableau610" displayName="Tableau610" ref="G20:I25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="G20:I25" xr:uid="{18208E07-AE00-42BB-B6B8-7046468EAA03}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{36809B6F-36E1-4201-B9CE-F32771FA12EA}" name="Observation" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{9CD5E82C-1995-4075-A6E8-31D19E8384F0}" name="Information parfaite" dataDxfId="1"/>
@@ -1641,7 +1641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BADBCD8-B019-405B-B880-05E3AEC9CA36}">
-  <dimension ref="B2:I59"/>
+  <dimension ref="B2:I57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
@@ -1656,7 +1656,7 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -1674,196 +1674,193 @@
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-    </row>
-    <row r="5" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-    </row>
-    <row r="6" spans="2:9" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
+    <row r="4" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="2:9" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="4">
+        <v>40</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0.36899999999999999</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0.92800000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="45" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="8">
+        <v>0.45800000000000002</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0.40699999999999997</v>
+      </c>
+      <c r="H7" s="8">
+        <v>0.97899999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0.4</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0.36899999999999999</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0.92800000000000005</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="4">
-        <v>24</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="E8" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8" s="8">
-        <v>0.45800000000000002</v>
+        <v>0.91700000000000004</v>
       </c>
       <c r="G8" s="8">
-        <v>0.40699999999999997</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="H8" s="8">
-        <v>0.97899999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="4">
-        <v>12</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="8">
-        <v>0.91700000000000004</v>
-      </c>
-      <c r="G9" s="8">
-        <v>0.49399999999999999</v>
-      </c>
-      <c r="H9" s="8">
         <v>0.995</v>
       </c>
     </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+    </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
@@ -1872,87 +1869,102 @@
       <c r="E18" s="4"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="13"/>
-      <c r="G20" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-    </row>
-    <row r="21" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
+      <c r="B19" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="13"/>
+      <c r="G19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+    </row>
+    <row r="20" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="G21" s="1" t="s">
+      <c r="E20" s="1"/>
+      <c r="G20" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="2">
+        <v>500</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="2">
+        <v>21</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
         <v>500</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="2">
+        <v>19</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="G22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="2">
-        <v>21</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B23" s="2">
-        <v>500</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="D23" s="2">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E23" s="2"/>
       <c r="G23" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
@@ -1960,468 +1972,437 @@
         <v>2000</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="D24" s="2">
         <v>11</v>
       </c>
       <c r="E24" s="2"/>
       <c r="G24" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B25" s="2">
         <v>2000</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D25" s="2">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E25" s="2"/>
       <c r="G25" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="2">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="D26" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E26" s="2"/>
-      <c r="G26" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
         <v>5000</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="D27" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E27" s="2"/>
     </row>
-    <row r="28" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B28" s="2">
-        <v>5000</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" s="2">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+    </row>
+    <row r="31" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+    </row>
+    <row r="33" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-    </row>
-    <row r="32" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="12"/>
-    </row>
-    <row r="33" spans="2:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
+      <c r="D33" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-    </row>
-    <row r="35" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G35" s="1" t="s">
+      <c r="B34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="4">
         <v>40</v>
       </c>
-      <c r="H35" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D34" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F34" s="6">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="G34" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="H34" s="7">
+        <v>0.23080000000000001</v>
+      </c>
+      <c r="I34" s="6">
+        <v>0.94199999999999995</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="4">
+        <v>24</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F35" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="G35" s="6">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="H35" s="7">
+        <v>0.31419999999999998</v>
+      </c>
+      <c r="I35" s="6">
+        <v>0.98599999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="45" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C36" s="4">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F36" s="6">
-        <v>0.72499999999999998</v>
+        <v>0.58299999999999996</v>
       </c>
       <c r="G36" s="6">
-        <v>0.25</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="H36" s="7">
-        <v>0.23080000000000001</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="I36" s="6">
-        <v>0.94199999999999995</v>
+        <v>0.96099999999999997</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="4">
-        <v>24</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F37" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="G37" s="6">
-        <v>0.20799999999999999</v>
-      </c>
-      <c r="H37" s="7">
-        <v>0.31419999999999998</v>
-      </c>
-      <c r="I37" s="6">
-        <v>0.98599999999999999</v>
-      </c>
-    </row>
-    <row r="38" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B38" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" s="4">
-        <v>12</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F38" s="6">
-        <v>0.58299999999999996</v>
-      </c>
-      <c r="G38" s="6">
-        <v>0.33300000000000002</v>
-      </c>
-      <c r="H38" s="7">
-        <v>0.33300000000000002</v>
-      </c>
-      <c r="I38" s="6">
-        <v>0.96099999999999997</v>
-      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="6"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="6"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="6"/>
+      <c r="B39" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="6"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E40" s="1" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B42" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B45" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E46" s="4" t="s">
         <v>72</v>
       </c>
     </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+    </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="B47" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B49" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
+      <c r="B49" s="4">
+        <v>500</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" s="4">
+        <v>15</v>
+      </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B50" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B50" s="4">
+        <v>500</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B51" s="4">
         <v>500</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D51" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B52" s="4">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="C52" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D52" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B53" s="4">
+        <v>2000</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D52" s="4">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="2:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="B53" s="4">
-        <v>500</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="D53" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B54" s="4">
         <v>2000</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D54" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B55" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="D55" s="4">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="56" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B56" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="D56" s="4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B57" s="4">
         <v>5000</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D57" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B58" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D58" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="59" spans="2:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="B59" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D59" s="4">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B32:I32"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>